<commit_message>
feat: make category strip fully dynamic and add image_id support to category admin form
</commit_message>
<xml_diff>
--- a/Silver_House_Production_Readiness_Checklist.xlsx
+++ b/Silver_House_Production_Readiness_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\E drive\SilverHouse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BAC937-EF19-4789-BCB5-B9CD072EDAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC90186D-0E2D-44FB-8668-D204B11AC9AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="148">
   <si>
     <t>SILVER HOUSE — PRODUCTION-GRADE E-COMMERCE ROADMAP &amp; AUDIT</t>
   </si>
@@ -471,14 +471,17 @@
     <t>Server maintenance policy needed on hosting provider</t>
   </si>
   <si>
+    <t>Pending</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve"> ❌ </t>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="9.5"/>
-        <color rgb="FFC00000"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
@@ -625,15 +628,15 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="9.5"/>
+      <color rgb="FF202124"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="9.5"/>
-      <color rgb="FFC00000"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9.5"/>
-      <color rgb="FF202124"/>
+      <color rgb="FF137333"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -715,7 +718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -777,6 +780,18 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -784,17 +799,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1111,26 +1117,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -1156,7 +1162,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIF(E8:E46, "*Completed*")</f>
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D5" s="8">
         <f>COUNTIF(E8:E46, "*In Progress*")</f>
@@ -1164,11 +1170,11 @@
       </c>
       <c r="E5" s="9">
         <f>COUNTIF(E7:E46, "*Pending*")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F5" s="10" t="str">
         <f>ROUND((COUNTIF(E8:E46,"*Completed*")/COUNTA(B8:B46))*100, 1) &amp; "%"</f>
-        <v>74.4%</v>
+        <v>61.5%</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1188,7 +1194,7 @@
       <c r="E7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="21" t="s">
         <v>12</v>
       </c>
       <c r="G7" s="12" t="s">
@@ -1208,7 +1214,7 @@
       <c r="D8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="23" t="s">
         <v>146</v>
       </c>
       <c r="F8" s="16" t="s">
@@ -1329,7 +1335,7 @@
       <c r="F13" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="24" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1461,7 +1467,7 @@
       <c r="D19" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="22" t="s">
         <v>55</v>
       </c>
       <c r="F19" s="17" t="s">
@@ -1691,8 +1697,8 @@
       <c r="D29" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>17</v>
+      <c r="E29" s="23" t="s">
+        <v>146</v>
       </c>
       <c r="F29" s="16" t="s">
         <v>18</v>
@@ -1714,8 +1720,8 @@
       <c r="D30" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E30" s="15" t="s">
-        <v>17</v>
+      <c r="E30" s="23" t="s">
+        <v>146</v>
       </c>
       <c r="F30" s="16" t="s">
         <v>18</v>
@@ -1737,8 +1743,8 @@
       <c r="D31" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="E31" s="15" t="s">
-        <v>17</v>
+      <c r="E31" s="23" t="s">
+        <v>146</v>
       </c>
       <c r="F31" s="16" t="s">
         <v>18</v>
@@ -1760,8 +1766,8 @@
       <c r="D32" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="E32" s="15" t="s">
-        <v>17</v>
+      <c r="E32" s="23" t="s">
+        <v>146</v>
       </c>
       <c r="F32" s="16" t="s">
         <v>18</v>
@@ -2036,8 +2042,8 @@
       <c r="D44" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="E44" s="15" t="s">
-        <v>17</v>
+      <c r="E44" s="28" t="s">
+        <v>147</v>
       </c>
       <c r="F44" s="17" t="s">
         <v>25</v>
@@ -2121,5 +2127,6 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>